<commit_message>
Update to SNES sheet
</commit_message>
<xml_diff>
--- a/snes/Every Snes Game (US_EU) - GMDQ.xlsx
+++ b/snes/Every Snes Game (US_EU) - GMDQ.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\2kgames.t2.corp\Network\2KGCZE\ToolTeam\Tableau\GitHub\103percent\GamesOnSpreadsheets\GamesOnSpreadsheets\snes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jak.Marshall\Documents\GitHub\GamesOnSpreadsheets\snes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF80F20E-F15D-4A78-9ECE-C72DC731D6E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{159F1105-69DC-47ED-ADD2-965327843A48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1365" yWindow="1650" windowWidth="35235" windowHeight="18300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4065" yWindow="2025" windowWidth="27870" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw Data" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2323" uniqueCount="1111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2329" uniqueCount="1113">
   <si>
     <t>Title</t>
   </si>
@@ -3354,6 +3354,12 @@
   </si>
   <si>
     <t>White Owl</t>
+  </si>
+  <si>
+    <t>Todd McFarlane's Spawn: The Video Game</t>
+  </si>
+  <si>
+    <t>Sunset Riders</t>
   </si>
 </sst>
 </file>
@@ -3647,7 +3653,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:D771"/>
+  <dimension ref="A1:D773"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="40.140625" customWidth="1"/>
@@ -11721,122 +11727,122 @@
     </row>
     <row r="577" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A577" s="2" t="s">
-        <v>863</v>
+        <v>1112</v>
       </c>
       <c r="B577" s="2">
-        <v>1994</v>
+        <v>1993</v>
       </c>
       <c r="C577" s="2" t="s">
-        <v>864</v>
+        <v>28</v>
       </c>
       <c r="D577" s="2" t="s">
-        <v>864</v>
+        <v>28</v>
       </c>
     </row>
     <row r="578" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A578" s="2" t="s">
-        <v>865</v>
+        <v>863</v>
       </c>
       <c r="B578" s="2">
-        <v>1992</v>
+        <v>1994</v>
       </c>
       <c r="C578" s="2" t="s">
-        <v>65</v>
+        <v>864</v>
       </c>
       <c r="D578" s="2" t="s">
-        <v>866</v>
+        <v>864</v>
       </c>
     </row>
     <row r="579" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A579" s="2" t="s">
-        <v>867</v>
+        <v>865</v>
       </c>
       <c r="B579" s="2">
-        <v>1995</v>
+        <v>1992</v>
       </c>
       <c r="C579" s="2" t="s">
         <v>65</v>
       </c>
       <c r="D579" s="2" t="s">
-        <v>868</v>
+        <v>866</v>
       </c>
     </row>
     <row r="580" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A580" s="2" t="s">
-        <v>869</v>
+        <v>867</v>
       </c>
       <c r="B580" s="2">
-        <v>1994</v>
+        <v>1995</v>
       </c>
       <c r="C580" s="2" t="s">
-        <v>52</v>
+        <v>65</v>
       </c>
       <c r="D580" s="2" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
     </row>
     <row r="581" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A581" s="2" t="s">
-        <v>871</v>
+        <v>869</v>
       </c>
       <c r="B581" s="2">
-        <v>1993</v>
+        <v>1994</v>
       </c>
       <c r="C581" s="2" t="s">
-        <v>508</v>
+        <v>52</v>
       </c>
       <c r="D581" s="2" t="s">
-        <v>872</v>
+        <v>870</v>
       </c>
     </row>
     <row r="582" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A582" s="2" t="s">
-        <v>873</v>
+        <v>871</v>
       </c>
       <c r="B582" s="2">
         <v>1993</v>
       </c>
       <c r="C582" s="2" t="s">
-        <v>119</v>
+        <v>508</v>
       </c>
       <c r="D582" s="2" t="s">
-        <v>87</v>
+        <v>872</v>
       </c>
     </row>
     <row r="583" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A583" s="2" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="B583" s="2">
-        <v>1991</v>
+        <v>1993</v>
       </c>
       <c r="C583" s="2" t="s">
-        <v>875</v>
+        <v>119</v>
       </c>
       <c r="D583" s="2" t="s">
-        <v>875</v>
+        <v>87</v>
       </c>
     </row>
     <row r="584" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A584" s="2" t="s">
-        <v>876</v>
+        <v>874</v>
       </c>
       <c r="B584" s="2">
         <v>1991</v>
       </c>
       <c r="C584" s="2" t="s">
-        <v>164</v>
+        <v>875</v>
       </c>
       <c r="D584" s="2" t="s">
-        <v>124</v>
+        <v>875</v>
       </c>
     </row>
     <row r="585" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A585" s="2" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="B585" s="2">
-        <v>1994</v>
+        <v>1991</v>
       </c>
       <c r="C585" s="2" t="s">
         <v>164</v>
@@ -11847,10 +11853,10 @@
     </row>
     <row r="586" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A586" s="2" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="B586" s="2">
-        <v>1995</v>
+        <v>1994</v>
       </c>
       <c r="C586" s="2" t="s">
         <v>164</v>
@@ -11861,94 +11867,94 @@
     </row>
     <row r="587" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A587" s="2" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="B587" s="2">
-        <v>1992</v>
+        <v>1995</v>
       </c>
       <c r="C587" s="2" t="s">
-        <v>12</v>
+        <v>164</v>
       </c>
       <c r="D587" s="2" t="s">
-        <v>12</v>
+        <v>124</v>
       </c>
     </row>
     <row r="588" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A588" s="2" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="B588" s="2">
-        <v>1993</v>
+        <v>1992</v>
       </c>
       <c r="C588" s="2" t="s">
-        <v>52</v>
+        <v>12</v>
       </c>
       <c r="D588" s="2" t="s">
-        <v>881</v>
+        <v>12</v>
       </c>
     </row>
     <row r="589" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A589" s="2" t="s">
-        <v>882</v>
+        <v>880</v>
       </c>
       <c r="B589" s="2">
-        <v>1992</v>
+        <v>1993</v>
       </c>
       <c r="C589" s="2" t="s">
-        <v>254</v>
+        <v>52</v>
       </c>
       <c r="D589" s="2" t="s">
-        <v>35</v>
+        <v>881</v>
       </c>
     </row>
     <row r="590" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A590" s="2" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="B590" s="2">
-        <v>1994</v>
+        <v>1992</v>
       </c>
       <c r="C590" s="2" t="s">
         <v>254</v>
       </c>
       <c r="D590" s="2" t="s">
-        <v>254</v>
+        <v>35</v>
       </c>
     </row>
     <row r="591" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A591" s="2" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="B591" s="2">
-        <v>1993</v>
+        <v>1994</v>
       </c>
       <c r="C591" s="2" t="s">
-        <v>885</v>
+        <v>254</v>
       </c>
       <c r="D591" s="2" t="s">
-        <v>106</v>
+        <v>254</v>
       </c>
     </row>
     <row r="592" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A592" s="2" t="s">
-        <v>886</v>
+        <v>884</v>
       </c>
       <c r="B592" s="2">
         <v>1993</v>
       </c>
       <c r="C592" s="2" t="s">
-        <v>65</v>
+        <v>885</v>
       </c>
       <c r="D592" s="2" t="s">
-        <v>866</v>
+        <v>106</v>
       </c>
     </row>
     <row r="593" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A593" s="2" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="B593" s="2">
-        <v>1994</v>
+        <v>1993</v>
       </c>
       <c r="C593" s="2" t="s">
         <v>65</v>
@@ -11959,332 +11965,332 @@
     </row>
     <row r="594" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A594" s="2" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="B594" s="2">
-        <v>1995</v>
+        <v>1994</v>
       </c>
       <c r="C594" s="2" t="s">
         <v>65</v>
       </c>
       <c r="D594" s="2" t="s">
-        <v>65</v>
+        <v>866</v>
       </c>
     </row>
     <row r="595" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A595" s="2" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="B595" s="2">
-        <v>1994</v>
+        <v>1995</v>
       </c>
       <c r="C595" s="2" t="s">
         <v>65</v>
       </c>
       <c r="D595" s="2" t="s">
-        <v>890</v>
+        <v>65</v>
       </c>
     </row>
     <row r="596" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A596" s="2" t="s">
-        <v>891</v>
+        <v>889</v>
       </c>
       <c r="B596" s="2">
-        <v>1992</v>
+        <v>1994</v>
       </c>
       <c r="C596" s="2" t="s">
-        <v>240</v>
+        <v>65</v>
       </c>
       <c r="D596" s="2" t="s">
-        <v>117</v>
+        <v>890</v>
       </c>
     </row>
     <row r="597" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A597" s="2" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="B597" s="2">
         <v>1992</v>
       </c>
       <c r="C597" s="2" t="s">
-        <v>55</v>
+        <v>240</v>
       </c>
       <c r="D597" s="2" t="s">
-        <v>55</v>
+        <v>117</v>
       </c>
     </row>
     <row r="598" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A598" s="2" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="B598" s="2">
-        <v>1993</v>
+        <v>1992</v>
       </c>
       <c r="C598" s="2" t="s">
-        <v>193</v>
+        <v>55</v>
       </c>
       <c r="D598" s="2" t="s">
-        <v>894</v>
+        <v>55</v>
       </c>
     </row>
     <row r="599" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A599" s="2" t="s">
-        <v>895</v>
+        <v>893</v>
       </c>
       <c r="B599" s="2">
-        <v>1991</v>
+        <v>1993</v>
       </c>
       <c r="C599" s="2" t="s">
-        <v>28</v>
+        <v>193</v>
       </c>
       <c r="D599" s="2" t="s">
-        <v>28</v>
+        <v>894</v>
       </c>
     </row>
     <row r="600" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A600" s="2" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="B600" s="2">
-        <v>1993</v>
+        <v>1991</v>
       </c>
       <c r="C600" s="2" t="s">
-        <v>84</v>
+        <v>28</v>
       </c>
       <c r="D600" s="2" t="s">
-        <v>84</v>
+        <v>28</v>
       </c>
     </row>
     <row r="601" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A601" s="2" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="B601" s="2">
         <v>1993</v>
       </c>
       <c r="C601" s="2" t="s">
-        <v>428</v>
+        <v>84</v>
       </c>
       <c r="D601" s="2" t="s">
-        <v>428</v>
+        <v>84</v>
       </c>
     </row>
     <row r="602" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A602" s="2" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="B602" s="2">
-        <v>1994</v>
+        <v>1993</v>
       </c>
       <c r="C602" s="2" t="s">
-        <v>193</v>
+        <v>428</v>
       </c>
       <c r="D602" s="2" t="s">
-        <v>899</v>
+        <v>428</v>
       </c>
     </row>
     <row r="603" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A603" s="2" t="s">
-        <v>900</v>
+        <v>898</v>
       </c>
       <c r="B603" s="2">
-        <v>1992</v>
+        <v>1994</v>
       </c>
       <c r="C603" s="2" t="s">
-        <v>119</v>
+        <v>193</v>
       </c>
       <c r="D603" s="2" t="s">
-        <v>240</v>
+        <v>899</v>
       </c>
     </row>
     <row r="604" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A604" s="2" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="B604" s="2">
-        <v>1995</v>
+        <v>1992</v>
       </c>
       <c r="C604" s="2" t="s">
-        <v>161</v>
+        <v>119</v>
       </c>
       <c r="D604" s="2" t="s">
-        <v>180</v>
+        <v>240</v>
       </c>
     </row>
     <row r="605" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A605" s="2" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="B605" s="2">
-        <v>1992</v>
+        <v>1995</v>
       </c>
       <c r="C605" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="D605" s="2" t="s">
-        <v>164</v>
+        <v>180</v>
       </c>
     </row>
     <row r="606" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A606" s="2" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="B606" s="2">
-        <v>1991</v>
+        <v>1992</v>
       </c>
       <c r="C606" s="2" t="s">
-        <v>55</v>
+        <v>164</v>
       </c>
       <c r="D606" s="2" t="s">
-        <v>55</v>
+        <v>164</v>
       </c>
     </row>
     <row r="607" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A607" s="2" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="B607" s="2">
-        <v>1994</v>
+        <v>1991</v>
       </c>
       <c r="C607" s="2" t="s">
-        <v>164</v>
+        <v>55</v>
       </c>
       <c r="D607" s="2" t="s">
-        <v>124</v>
+        <v>55</v>
       </c>
     </row>
     <row r="608" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A608" s="2" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="B608" s="2">
         <v>1994</v>
       </c>
       <c r="C608" s="2" t="s">
-        <v>567</v>
+        <v>164</v>
       </c>
       <c r="D608" s="2" t="s">
-        <v>567</v>
+        <v>124</v>
       </c>
     </row>
     <row r="609" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A609" s="2" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="B609" s="2">
-        <v>1993</v>
+        <v>1994</v>
       </c>
       <c r="C609" s="2" t="s">
-        <v>108</v>
+        <v>567</v>
       </c>
       <c r="D609" s="2" t="s">
-        <v>44</v>
+        <v>567</v>
       </c>
     </row>
     <row r="610" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A610" s="2" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="B610" s="2">
-        <v>1994</v>
+        <v>1993</v>
       </c>
       <c r="C610" s="2" t="s">
-        <v>19</v>
+        <v>108</v>
       </c>
       <c r="D610" s="2" t="s">
-        <v>908</v>
+        <v>44</v>
       </c>
     </row>
     <row r="611" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A611" s="2" t="s">
-        <v>909</v>
+        <v>907</v>
       </c>
       <c r="B611" s="2">
         <v>1994</v>
       </c>
       <c r="C611" s="2" t="s">
-        <v>83</v>
+        <v>19</v>
       </c>
       <c r="D611" s="2" t="s">
-        <v>221</v>
+        <v>908</v>
       </c>
     </row>
     <row r="612" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A612" s="2" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="B612" s="2">
-        <v>1993</v>
+        <v>1994</v>
       </c>
       <c r="C612" s="2" t="s">
-        <v>808</v>
+        <v>83</v>
       </c>
       <c r="D612" s="2" t="s">
-        <v>808</v>
+        <v>221</v>
       </c>
     </row>
     <row r="613" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A613" s="2" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="B613" s="2">
         <v>1993</v>
       </c>
       <c r="C613" s="2" t="s">
-        <v>83</v>
+        <v>808</v>
       </c>
       <c r="D613" s="2" t="s">
-        <v>688</v>
+        <v>808</v>
       </c>
     </row>
     <row r="614" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A614" s="2" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="B614" s="2">
-        <v>1992</v>
+        <v>1993</v>
       </c>
       <c r="C614" s="2" t="s">
         <v>83</v>
       </c>
       <c r="D614" s="2" t="s">
-        <v>83</v>
+        <v>688</v>
       </c>
     </row>
     <row r="615" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A615" s="2" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="B615" s="2">
-        <v>1996</v>
+        <v>1992</v>
       </c>
       <c r="C615" s="2" t="s">
         <v>83</v>
       </c>
       <c r="D615" s="2" t="s">
-        <v>169</v>
+        <v>83</v>
       </c>
     </row>
     <row r="616" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A616" s="2" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B616" s="2">
-        <v>1991</v>
+        <v>1996</v>
       </c>
       <c r="C616" s="2" t="s">
         <v>83</v>
       </c>
       <c r="D616" s="2" t="s">
-        <v>83</v>
+        <v>169</v>
       </c>
     </row>
     <row r="617" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A617" s="2" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="B617" s="2">
-        <v>1995</v>
+        <v>1991</v>
       </c>
       <c r="C617" s="2" t="s">
         <v>83</v>
@@ -12295,10 +12301,10 @@
     </row>
     <row r="618" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A618" s="2" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="B618" s="2">
-        <v>1994</v>
+        <v>1995</v>
       </c>
       <c r="C618" s="2" t="s">
         <v>83</v>
@@ -12309,66 +12315,66 @@
     </row>
     <row r="619" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A619" s="2" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="B619" s="2">
-        <v>1993</v>
+        <v>1994</v>
       </c>
       <c r="C619" s="2" t="s">
-        <v>5</v>
+        <v>83</v>
       </c>
       <c r="D619" s="2" t="s">
-        <v>918</v>
+        <v>83</v>
       </c>
     </row>
     <row r="620" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A620" s="2" t="s">
-        <v>919</v>
+        <v>917</v>
       </c>
       <c r="B620" s="2">
         <v>1993</v>
       </c>
       <c r="C620" s="2" t="s">
-        <v>875</v>
+        <v>5</v>
       </c>
       <c r="D620" s="2" t="s">
-        <v>875</v>
+        <v>918</v>
       </c>
     </row>
     <row r="621" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A621" s="2" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="B621" s="2">
         <v>1993</v>
       </c>
       <c r="C621" s="2" t="s">
-        <v>84</v>
+        <v>875</v>
       </c>
       <c r="D621" s="2" t="s">
-        <v>84</v>
+        <v>875</v>
       </c>
     </row>
     <row r="622" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A622" s="2" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="B622" s="2">
-        <v>1992</v>
+        <v>1993</v>
       </c>
       <c r="C622" s="2" t="s">
-        <v>119</v>
+        <v>84</v>
       </c>
       <c r="D622" s="2" t="s">
-        <v>99</v>
+        <v>84</v>
       </c>
     </row>
     <row r="623" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A623" s="2" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="B623" s="2">
-        <v>1993</v>
+        <v>1992</v>
       </c>
       <c r="C623" s="2" t="s">
         <v>119</v>
@@ -12379,119 +12385,119 @@
     </row>
     <row r="624" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A624" s="2" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="B624" s="2">
-        <v>1994</v>
+        <v>1993</v>
       </c>
       <c r="C624" s="2" t="s">
-        <v>83</v>
+        <v>119</v>
       </c>
       <c r="D624" s="2" t="s">
-        <v>924</v>
+        <v>99</v>
       </c>
     </row>
     <row r="625" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A625" s="2" t="s">
-        <v>925</v>
+        <v>923</v>
       </c>
       <c r="B625" s="2">
-        <v>1992</v>
+        <v>1994</v>
       </c>
       <c r="C625" s="2" t="s">
         <v>83</v>
       </c>
       <c r="D625" s="2" t="s">
-        <v>124</v>
+        <v>924</v>
       </c>
     </row>
     <row r="626" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A626" s="2" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="B626" s="2">
-        <v>1993</v>
+        <v>1992</v>
       </c>
       <c r="C626" s="2" t="s">
-        <v>364</v>
+        <v>83</v>
       </c>
       <c r="D626" s="2" t="s">
-        <v>732</v>
+        <v>124</v>
       </c>
     </row>
     <row r="627" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A627" s="2" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="B627" s="2">
-        <v>1994</v>
+        <v>1993</v>
       </c>
       <c r="C627" s="2" t="s">
-        <v>83</v>
+        <v>364</v>
       </c>
       <c r="D627" s="2" t="s">
-        <v>928</v>
+        <v>732</v>
       </c>
     </row>
     <row r="628" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A628" s="2" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
       <c r="B628" s="2">
-        <v>1995</v>
+        <v>1994</v>
       </c>
       <c r="C628" s="2" t="s">
-        <v>477</v>
+        <v>83</v>
       </c>
       <c r="D628" s="2" t="s">
-        <v>152</v>
+        <v>928</v>
       </c>
     </row>
     <row r="629" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A629" s="2" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="B629" s="2">
-        <v>1991</v>
+        <v>1995</v>
       </c>
       <c r="C629" s="2" t="s">
-        <v>268</v>
+        <v>477</v>
       </c>
       <c r="D629" s="2" t="s">
-        <v>268</v>
+        <v>152</v>
       </c>
     </row>
     <row r="630" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A630" s="2" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="B630" s="2">
-        <v>1992</v>
+        <v>1991</v>
       </c>
       <c r="C630" s="2" t="s">
-        <v>83</v>
+        <v>268</v>
       </c>
       <c r="D630" s="2" t="s">
-        <v>83</v>
+        <v>268</v>
       </c>
     </row>
     <row r="631" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A631" s="2" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="B631" s="2">
-        <v>1993</v>
+        <v>1992</v>
       </c>
       <c r="C631" s="2" t="s">
-        <v>193</v>
+        <v>83</v>
       </c>
       <c r="D631" s="2" t="s">
-        <v>210</v>
+        <v>83</v>
       </c>
     </row>
     <row r="632" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A632" s="2" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="B632" s="2">
         <v>1993</v>
@@ -12500,85 +12506,85 @@
         <v>193</v>
       </c>
       <c r="D632" s="2" t="s">
-        <v>934</v>
+        <v>210</v>
       </c>
     </row>
     <row r="633" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A633" s="2" t="s">
-        <v>935</v>
+        <v>933</v>
       </c>
       <c r="B633" s="2">
-        <v>1992</v>
+        <v>1993</v>
       </c>
       <c r="C633" s="2" t="s">
-        <v>108</v>
+        <v>193</v>
       </c>
       <c r="D633" s="2" t="s">
-        <v>221</v>
+        <v>934</v>
       </c>
     </row>
     <row r="634" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A634" s="2" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="B634" s="2">
         <v>1992</v>
       </c>
       <c r="C634" s="2" t="s">
-        <v>83</v>
+        <v>108</v>
       </c>
       <c r="D634" s="2" t="s">
-        <v>327</v>
+        <v>221</v>
       </c>
     </row>
     <row r="635" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A635" s="2" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="B635" s="2">
         <v>1992</v>
       </c>
       <c r="C635" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D635" s="2" t="s">
-        <v>84</v>
+        <v>327</v>
       </c>
     </row>
     <row r="636" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A636" s="2" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="B636" s="2">
-        <v>1994</v>
+        <v>1992</v>
       </c>
       <c r="C636" s="2" t="s">
-        <v>220</v>
+        <v>84</v>
       </c>
       <c r="D636" s="2" t="s">
-        <v>220</v>
+        <v>84</v>
       </c>
     </row>
     <row r="637" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A637" s="2" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="B637" s="2">
-        <v>1992</v>
+        <v>1994</v>
       </c>
       <c r="C637" s="2" t="s">
-        <v>434</v>
+        <v>220</v>
       </c>
       <c r="D637" s="2" t="s">
-        <v>204</v>
+        <v>220</v>
       </c>
     </row>
     <row r="638" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A638" s="2" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="B638" s="2">
-        <v>1993</v>
+        <v>1992</v>
       </c>
       <c r="C638" s="2" t="s">
         <v>434</v>
@@ -12589,10 +12595,10 @@
     </row>
     <row r="639" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A639" s="2" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="B639" s="2">
-        <v>1994</v>
+        <v>1993</v>
       </c>
       <c r="C639" s="2" t="s">
         <v>434</v>
@@ -12603,83 +12609,83 @@
     </row>
     <row r="640" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A640" s="2" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="B640" s="2">
         <v>1994</v>
       </c>
       <c r="C640" s="2" t="s">
-        <v>55</v>
+        <v>434</v>
       </c>
       <c r="D640" s="2" t="s">
-        <v>55</v>
+        <v>204</v>
       </c>
     </row>
     <row r="641" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A641" s="2" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="B641" s="2">
-        <v>1993</v>
+        <v>1994</v>
       </c>
       <c r="C641" s="2" t="s">
-        <v>944</v>
+        <v>55</v>
       </c>
       <c r="D641" s="2" t="s">
-        <v>944</v>
+        <v>55</v>
       </c>
     </row>
     <row r="642" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A642" s="2" t="s">
-        <v>945</v>
+        <v>943</v>
       </c>
       <c r="B642" s="2">
-        <v>1991</v>
+        <v>1993</v>
       </c>
       <c r="C642" s="2" t="s">
-        <v>83</v>
+        <v>944</v>
       </c>
       <c r="D642" s="2" t="s">
-        <v>946</v>
+        <v>944</v>
       </c>
     </row>
     <row r="643" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A643" s="2" t="s">
-        <v>947</v>
+        <v>945</v>
       </c>
       <c r="B643" s="2">
-        <v>1994</v>
+        <v>1991</v>
       </c>
       <c r="C643" s="2" t="s">
-        <v>808</v>
+        <v>83</v>
       </c>
       <c r="D643" s="2" t="s">
-        <v>294</v>
+        <v>946</v>
       </c>
     </row>
     <row r="644" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A644" s="2" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="B644" s="2">
-        <v>1993</v>
+        <v>1994</v>
       </c>
       <c r="C644" s="2" t="s">
-        <v>508</v>
+        <v>808</v>
       </c>
       <c r="D644" s="2" t="s">
-        <v>435</v>
+        <v>294</v>
       </c>
     </row>
     <row r="645" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A645" s="2" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="B645" s="2">
-        <v>1995</v>
+        <v>1993</v>
       </c>
       <c r="C645" s="2" t="s">
-        <v>11</v>
+        <v>508</v>
       </c>
       <c r="D645" s="2" t="s">
         <v>435</v>
@@ -12687,21 +12693,21 @@
     </row>
     <row r="646" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A646" s="2" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="B646" s="2">
-        <v>1993</v>
+        <v>1995</v>
       </c>
       <c r="C646" s="2" t="s">
-        <v>148</v>
+        <v>11</v>
       </c>
       <c r="D646" s="2" t="s">
-        <v>951</v>
+        <v>435</v>
       </c>
     </row>
     <row r="647" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A647" s="2" t="s">
-        <v>952</v>
+        <v>950</v>
       </c>
       <c r="B647" s="2">
         <v>1993</v>
@@ -12710,113 +12716,113 @@
         <v>148</v>
       </c>
       <c r="D647" s="2" t="s">
-        <v>148</v>
+        <v>951</v>
       </c>
     </row>
     <row r="648" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A648" s="2" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="B648" s="2">
-        <v>1994</v>
+        <v>1993</v>
       </c>
       <c r="C648" s="2" t="s">
-        <v>12</v>
+        <v>148</v>
       </c>
       <c r="D648" s="2" t="s">
-        <v>12</v>
+        <v>148</v>
       </c>
     </row>
     <row r="649" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A649" s="2" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="B649" s="2">
-        <v>1995</v>
+        <v>1994</v>
       </c>
       <c r="C649" s="2" t="s">
-        <v>65</v>
+        <v>12</v>
       </c>
       <c r="D649" s="2" t="s">
-        <v>438</v>
+        <v>12</v>
       </c>
     </row>
     <row r="650" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A650" s="2" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
       <c r="B650" s="2">
         <v>1995</v>
       </c>
       <c r="C650" s="2" t="s">
-        <v>11</v>
+        <v>65</v>
       </c>
       <c r="D650" s="2" t="s">
-        <v>709</v>
+        <v>438</v>
       </c>
     </row>
     <row r="651" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A651" s="2" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="B651" s="2">
-        <v>1993</v>
+        <v>1995</v>
       </c>
       <c r="C651" s="2" t="s">
-        <v>957</v>
+        <v>11</v>
       </c>
       <c r="D651" s="2" t="s">
-        <v>84</v>
+        <v>709</v>
       </c>
     </row>
     <row r="652" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A652" s="2" t="s">
-        <v>958</v>
+        <v>956</v>
       </c>
       <c r="B652" s="2">
         <v>1993</v>
       </c>
       <c r="C652" s="2" t="s">
-        <v>431</v>
+        <v>957</v>
       </c>
       <c r="D652" s="2" t="s">
-        <v>20</v>
+        <v>84</v>
       </c>
     </row>
     <row r="653" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A653" s="2" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
       <c r="B653" s="2">
         <v>1993</v>
       </c>
       <c r="C653" s="2" t="s">
-        <v>19</v>
+        <v>431</v>
       </c>
       <c r="D653" s="2" t="s">
-        <v>228</v>
+        <v>20</v>
       </c>
     </row>
     <row r="654" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A654" s="2" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="B654" s="2">
-        <v>1994</v>
+        <v>1993</v>
       </c>
       <c r="C654" s="2" t="s">
-        <v>644</v>
+        <v>19</v>
       </c>
       <c r="D654" s="2" t="s">
-        <v>644</v>
+        <v>228</v>
       </c>
     </row>
     <row r="655" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A655" s="2" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
       <c r="B655" s="2">
-        <v>1993</v>
+        <v>1994</v>
       </c>
       <c r="C655" s="2" t="s">
         <v>644</v>
@@ -12827,10 +12833,10 @@
     </row>
     <row r="656" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A656" s="2" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
       <c r="B656" s="2">
-        <v>1995</v>
+        <v>1993</v>
       </c>
       <c r="C656" s="2" t="s">
         <v>644</v>
@@ -12841,7 +12847,7 @@
     </row>
     <row r="657" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A657" s="2" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="B657" s="2">
         <v>1995</v>
@@ -12855,10 +12861,10 @@
     </row>
     <row r="658" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A658" s="2" t="s">
-        <v>964</v>
+        <v>963</v>
       </c>
       <c r="B658" s="2">
-        <v>1993</v>
+        <v>1995</v>
       </c>
       <c r="C658" s="2" t="s">
         <v>644</v>
@@ -12869,24 +12875,24 @@
     </row>
     <row r="659" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A659" s="2" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
       <c r="B659" s="2">
-        <v>1992</v>
+        <v>1993</v>
       </c>
       <c r="C659" s="2" t="s">
-        <v>28</v>
+        <v>644</v>
       </c>
       <c r="D659" s="2" t="s">
-        <v>28</v>
+        <v>644</v>
       </c>
     </row>
     <row r="660" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A660" s="2" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
       <c r="B660" s="2">
-        <v>1993</v>
+        <v>1992</v>
       </c>
       <c r="C660" s="2" t="s">
         <v>28</v>
@@ -12897,63 +12903,63 @@
     </row>
     <row r="661" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A661" s="2" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="B661" s="2">
         <v>1993</v>
       </c>
       <c r="C661" s="2" t="s">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="D661" s="2" t="s">
-        <v>52</v>
+        <v>28</v>
       </c>
     </row>
     <row r="662" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A662" s="2" t="s">
-        <v>968</v>
+        <v>967</v>
       </c>
       <c r="B662" s="2">
         <v>1993</v>
       </c>
       <c r="C662" s="2" t="s">
-        <v>431</v>
+        <v>52</v>
       </c>
       <c r="D662" s="2" t="s">
-        <v>395</v>
+        <v>52</v>
       </c>
     </row>
     <row r="663" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A663" s="2" t="s">
-        <v>969</v>
+        <v>968</v>
       </c>
       <c r="B663" s="2">
-        <v>1996</v>
+        <v>1993</v>
       </c>
       <c r="C663" s="2" t="s">
-        <v>83</v>
+        <v>431</v>
       </c>
       <c r="D663" s="2" t="s">
-        <v>22</v>
+        <v>395</v>
       </c>
     </row>
     <row r="664" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A664" s="2" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
       <c r="B664" s="2">
-        <v>1994</v>
+        <v>1996</v>
       </c>
       <c r="C664" s="2" t="s">
         <v>83</v>
       </c>
       <c r="D664" s="2" t="s">
-        <v>124</v>
+        <v>22</v>
       </c>
     </row>
     <row r="665" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A665" s="2" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
       <c r="B665" s="2">
         <v>1994</v>
@@ -12962,183 +12968,183 @@
         <v>83</v>
       </c>
       <c r="D665" s="2" t="s">
-        <v>336</v>
+        <v>124</v>
       </c>
     </row>
     <row r="666" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A666" s="2" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
       <c r="B666" s="2">
-        <v>1996</v>
+        <v>1994</v>
       </c>
       <c r="C666" s="2" t="s">
         <v>83</v>
       </c>
       <c r="D666" s="2" t="s">
-        <v>973</v>
+        <v>336</v>
       </c>
     </row>
     <row r="667" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A667" s="2" t="s">
-        <v>974</v>
+        <v>972</v>
       </c>
       <c r="B667" s="2">
         <v>1996</v>
       </c>
       <c r="C667" s="2" t="s">
-        <v>141</v>
+        <v>83</v>
       </c>
       <c r="D667" s="2" t="s">
-        <v>709</v>
+        <v>973</v>
       </c>
     </row>
     <row r="668" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A668" s="2" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
       <c r="B668" s="2">
         <v>1996</v>
       </c>
       <c r="C668" s="2" t="s">
-        <v>34</v>
+        <v>141</v>
       </c>
       <c r="D668" s="2" t="s">
-        <v>99</v>
+        <v>709</v>
       </c>
     </row>
     <row r="669" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A669" s="2" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="B669" s="2">
-        <v>1992</v>
+        <v>1996</v>
       </c>
       <c r="C669" s="2" t="s">
-        <v>508</v>
+        <v>34</v>
       </c>
       <c r="D669" s="2" t="s">
-        <v>977</v>
+        <v>99</v>
       </c>
     </row>
     <row r="670" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A670" s="2" t="s">
-        <v>978</v>
+        <v>976</v>
       </c>
       <c r="B670" s="2">
-        <v>1994</v>
+        <v>1992</v>
       </c>
       <c r="C670" s="2" t="s">
-        <v>672</v>
+        <v>508</v>
       </c>
       <c r="D670" s="2" t="s">
-        <v>99</v>
+        <v>977</v>
       </c>
     </row>
     <row r="671" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A671" s="2" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
       <c r="B671" s="2">
-        <v>1993</v>
+        <v>1994</v>
       </c>
       <c r="C671" s="2" t="s">
-        <v>428</v>
+        <v>672</v>
       </c>
       <c r="D671" s="2" t="s">
-        <v>359</v>
+        <v>99</v>
       </c>
     </row>
     <row r="672" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A672" s="2" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="B672" s="2">
-        <v>1994</v>
+        <v>1993</v>
       </c>
       <c r="C672" s="2" t="s">
-        <v>102</v>
+        <v>428</v>
       </c>
       <c r="D672" s="2" t="s">
-        <v>102</v>
+        <v>359</v>
       </c>
     </row>
     <row r="673" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A673" s="2" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="B673" s="2">
-        <v>1995</v>
+        <v>1994</v>
       </c>
       <c r="C673" s="2" t="s">
-        <v>135</v>
+        <v>102</v>
       </c>
       <c r="D673" s="2" t="s">
-        <v>899</v>
+        <v>102</v>
       </c>
     </row>
     <row r="674" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A674" s="2" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
       <c r="B674" s="2">
-        <v>1997</v>
+        <v>1995</v>
       </c>
       <c r="C674" s="2" t="s">
-        <v>34</v>
+        <v>135</v>
       </c>
       <c r="D674" s="2" t="s">
-        <v>983</v>
+        <v>899</v>
       </c>
     </row>
     <row r="675" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A675" s="2" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="B675" s="2">
-        <v>1994</v>
+        <v>1997</v>
       </c>
       <c r="C675" s="2" t="s">
-        <v>83</v>
+        <v>34</v>
       </c>
       <c r="D675" s="2" t="s">
-        <v>99</v>
+        <v>983</v>
       </c>
     </row>
     <row r="676" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A676" s="2" t="s">
-        <v>985</v>
+        <v>984</v>
       </c>
       <c r="B676" s="2">
-        <v>1995</v>
+        <v>1994</v>
       </c>
       <c r="C676" s="2" t="s">
-        <v>37</v>
+        <v>83</v>
       </c>
       <c r="D676" s="2" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
     </row>
     <row r="677" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A677" s="2" t="s">
-        <v>986</v>
+        <v>985</v>
       </c>
       <c r="B677" s="2">
-        <v>1993</v>
+        <v>1995</v>
       </c>
       <c r="C677" s="2" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="D677" s="2" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
     </row>
     <row r="678" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A678" s="2" t="s">
-        <v>987</v>
+        <v>986</v>
       </c>
       <c r="B678" s="2">
-        <v>1994</v>
+        <v>1993</v>
       </c>
       <c r="C678" s="2" t="s">
         <v>28</v>
@@ -13149,108 +13155,108 @@
     </row>
     <row r="679" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A679" s="2" t="s">
-        <v>988</v>
+        <v>987</v>
       </c>
       <c r="B679" s="2">
-        <v>1992</v>
+        <v>1994</v>
       </c>
       <c r="C679" s="2" t="s">
-        <v>989</v>
+        <v>28</v>
       </c>
       <c r="D679" s="2" t="s">
-        <v>322</v>
+        <v>28</v>
       </c>
     </row>
     <row r="680" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A680" s="2" t="s">
-        <v>990</v>
+        <v>988</v>
       </c>
       <c r="B680" s="2">
-        <v>1994</v>
+        <v>1992</v>
       </c>
       <c r="C680" s="2" t="s">
-        <v>808</v>
+        <v>989</v>
       </c>
       <c r="D680" s="2" t="s">
-        <v>991</v>
+        <v>322</v>
       </c>
     </row>
     <row r="681" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A681" s="2" t="s">
-        <v>992</v>
+        <v>990</v>
       </c>
       <c r="B681" s="2">
-        <v>1993</v>
+        <v>1994</v>
       </c>
       <c r="C681" s="2" t="s">
-        <v>405</v>
+        <v>808</v>
       </c>
       <c r="D681" s="2" t="s">
-        <v>130</v>
+        <v>991</v>
       </c>
     </row>
     <row r="682" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A682" s="2" t="s">
-        <v>993</v>
+        <v>1111</v>
       </c>
       <c r="B682" s="2">
-        <v>1994</v>
+        <v>1995</v>
       </c>
       <c r="C682" s="2" t="s">
-        <v>994</v>
+        <v>108</v>
       </c>
       <c r="D682" s="2" t="s">
-        <v>442</v>
+        <v>416</v>
       </c>
     </row>
     <row r="683" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A683" s="2" t="s">
-        <v>995</v>
+        <v>992</v>
       </c>
       <c r="B683" s="2">
         <v>1993</v>
       </c>
       <c r="C683" s="2" t="s">
-        <v>132</v>
+        <v>405</v>
       </c>
       <c r="D683" s="2" t="s">
-        <v>204</v>
+        <v>130</v>
       </c>
     </row>
     <row r="684" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A684" s="2" t="s">
-        <v>996</v>
+        <v>993</v>
       </c>
       <c r="B684" s="2">
-        <v>1992</v>
+        <v>1994</v>
       </c>
       <c r="C684" s="2" t="s">
-        <v>294</v>
+        <v>994</v>
       </c>
       <c r="D684" s="2" t="s">
-        <v>642</v>
+        <v>442</v>
       </c>
     </row>
     <row r="685" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A685" s="2" t="s">
-        <v>997</v>
+        <v>995</v>
       </c>
       <c r="B685" s="2">
         <v>1993</v>
       </c>
       <c r="C685" s="2" t="s">
-        <v>294</v>
+        <v>132</v>
       </c>
       <c r="D685" s="2" t="s">
-        <v>642</v>
+        <v>204</v>
       </c>
     </row>
     <row r="686" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A686" s="2" t="s">
-        <v>998</v>
+        <v>996</v>
       </c>
       <c r="B686" s="2">
-        <v>1995</v>
+        <v>1992</v>
       </c>
       <c r="C686" s="2" t="s">
         <v>294</v>
@@ -13261,111 +13267,111 @@
     </row>
     <row r="687" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A687" s="2" t="s">
-        <v>999</v>
+        <v>997</v>
       </c>
       <c r="B687" s="2">
         <v>1993</v>
       </c>
       <c r="C687" s="2" t="s">
-        <v>102</v>
+        <v>294</v>
       </c>
       <c r="D687" s="2" t="s">
-        <v>236</v>
+        <v>642</v>
       </c>
     </row>
     <row r="688" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A688" s="2" t="s">
-        <v>1000</v>
+        <v>998</v>
       </c>
       <c r="B688" s="2">
         <v>1995</v>
       </c>
       <c r="C688" s="2" t="s">
-        <v>695</v>
+        <v>294</v>
       </c>
       <c r="D688" s="2" t="s">
-        <v>586</v>
+        <v>642</v>
       </c>
     </row>
     <row r="689" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A689" s="2" t="s">
-        <v>1001</v>
+        <v>999</v>
       </c>
       <c r="B689" s="2">
         <v>1993</v>
       </c>
       <c r="C689" s="2" t="s">
-        <v>254</v>
+        <v>102</v>
       </c>
       <c r="D689" s="2" t="s">
-        <v>35</v>
+        <v>236</v>
       </c>
     </row>
     <row r="690" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A690" s="2" t="s">
-        <v>1002</v>
+        <v>1000</v>
       </c>
       <c r="B690" s="2">
-        <v>1993</v>
+        <v>1995</v>
       </c>
       <c r="C690" s="2" t="s">
-        <v>508</v>
+        <v>695</v>
       </c>
       <c r="D690" s="2" t="s">
-        <v>1003</v>
+        <v>586</v>
       </c>
     </row>
     <row r="691" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A691" s="2" t="s">
-        <v>1004</v>
+        <v>1001</v>
       </c>
       <c r="B691" s="2">
-        <v>1994</v>
+        <v>1993</v>
       </c>
       <c r="C691" s="2" t="s">
-        <v>119</v>
+        <v>254</v>
       </c>
       <c r="D691" s="2" t="s">
-        <v>119</v>
+        <v>35</v>
       </c>
     </row>
     <row r="692" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A692" s="2" t="s">
-        <v>1005</v>
+        <v>1002</v>
       </c>
       <c r="B692" s="2">
         <v>1993</v>
       </c>
       <c r="C692" s="2" t="s">
-        <v>336</v>
+        <v>508</v>
       </c>
       <c r="D692" s="2" t="s">
-        <v>1006</v>
+        <v>1003</v>
       </c>
     </row>
     <row r="693" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A693" s="2" t="s">
-        <v>1007</v>
+        <v>1004</v>
       </c>
       <c r="B693" s="2">
-        <v>1992</v>
+        <v>1994</v>
       </c>
       <c r="C693" s="2" t="s">
-        <v>1006</v>
+        <v>119</v>
       </c>
       <c r="D693" s="2" t="s">
-        <v>1006</v>
+        <v>119</v>
       </c>
     </row>
     <row r="694" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A694" s="2" t="s">
-        <v>1008</v>
+        <v>1005</v>
       </c>
       <c r="B694" s="2">
-        <v>1991</v>
+        <v>1993</v>
       </c>
       <c r="C694" s="2" t="s">
-        <v>1006</v>
+        <v>336</v>
       </c>
       <c r="D694" s="2" t="s">
         <v>1006</v>
@@ -13373,91 +13379,91 @@
     </row>
     <row r="695" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A695" s="2" t="s">
-        <v>1009</v>
+        <v>1007</v>
       </c>
       <c r="B695" s="2">
-        <v>1995</v>
+        <v>1992</v>
       </c>
       <c r="C695" s="2" t="s">
-        <v>431</v>
+        <v>1006</v>
       </c>
       <c r="D695" s="2" t="s">
-        <v>221</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="696" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A696" s="2" t="s">
-        <v>1010</v>
+        <v>1008</v>
       </c>
       <c r="B696" s="2">
-        <v>1993</v>
+        <v>1991</v>
       </c>
       <c r="C696" s="2" t="s">
-        <v>164</v>
+        <v>1006</v>
       </c>
       <c r="D696" s="2" t="s">
-        <v>164</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="697" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A697" s="2" t="s">
-        <v>1011</v>
+        <v>1009</v>
       </c>
       <c r="B697" s="2">
-        <v>1994</v>
+        <v>1995</v>
       </c>
       <c r="C697" s="2" t="s">
-        <v>254</v>
+        <v>431</v>
       </c>
       <c r="D697" s="2" t="s">
-        <v>254</v>
+        <v>221</v>
       </c>
     </row>
     <row r="698" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A698" s="2" t="s">
-        <v>1012</v>
+        <v>1010</v>
       </c>
       <c r="B698" s="2">
-        <v>1994</v>
+        <v>1993</v>
       </c>
       <c r="C698" s="2" t="s">
-        <v>336</v>
+        <v>164</v>
       </c>
       <c r="D698" s="2" t="s">
-        <v>1013</v>
+        <v>164</v>
       </c>
     </row>
     <row r="699" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A699" s="2" t="s">
-        <v>1014</v>
+        <v>1011</v>
       </c>
       <c r="B699" s="2">
         <v>1994</v>
       </c>
       <c r="C699" s="2" t="s">
-        <v>579</v>
+        <v>254</v>
       </c>
       <c r="D699" s="2" t="s">
-        <v>580</v>
+        <v>254</v>
       </c>
     </row>
     <row r="700" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A700" s="2" t="s">
-        <v>1015</v>
+        <v>1012</v>
       </c>
       <c r="B700" s="2">
         <v>1994</v>
       </c>
       <c r="C700" s="2" t="s">
-        <v>579</v>
+        <v>336</v>
       </c>
       <c r="D700" s="2" t="s">
-        <v>1016</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="701" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A701" s="2" t="s">
-        <v>1017</v>
+        <v>1014</v>
       </c>
       <c r="B701" s="2">
         <v>1994</v>
@@ -13471,797 +13477,797 @@
     </row>
     <row r="702" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A702" s="2" t="s">
-        <v>1018</v>
+        <v>1015</v>
       </c>
       <c r="B702" s="2">
         <v>1994</v>
       </c>
       <c r="C702" s="2" t="s">
-        <v>875</v>
+        <v>579</v>
       </c>
       <c r="D702" s="2" t="s">
-        <v>875</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="703" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A703" s="2" t="s">
-        <v>1019</v>
+        <v>1017</v>
       </c>
       <c r="B703" s="2">
-        <v>1996</v>
+        <v>1994</v>
       </c>
       <c r="C703" s="2" t="s">
-        <v>1020</v>
+        <v>579</v>
       </c>
       <c r="D703" s="2" t="s">
-        <v>1021</v>
+        <v>580</v>
       </c>
     </row>
     <row r="704" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A704" s="2" t="s">
-        <v>1022</v>
+        <v>1018</v>
       </c>
       <c r="B704" s="2">
-        <v>1991</v>
+        <v>1994</v>
       </c>
       <c r="C704" s="2" t="s">
-        <v>123</v>
+        <v>875</v>
       </c>
       <c r="D704" s="2" t="s">
-        <v>221</v>
+        <v>875</v>
       </c>
     </row>
     <row r="705" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A705" s="2" t="s">
-        <v>1023</v>
+        <v>1019</v>
       </c>
       <c r="B705" s="2">
-        <v>1993</v>
+        <v>1996</v>
       </c>
       <c r="C705" s="2" t="s">
-        <v>47</v>
+        <v>1020</v>
       </c>
       <c r="D705" s="2" t="s">
-        <v>47</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="706" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A706" s="2" t="s">
-        <v>1024</v>
+        <v>1022</v>
       </c>
       <c r="B706" s="2">
-        <v>1994</v>
+        <v>1991</v>
       </c>
       <c r="C706" s="2" t="s">
-        <v>47</v>
+        <v>123</v>
       </c>
       <c r="D706" s="2" t="s">
-        <v>47</v>
+        <v>221</v>
       </c>
     </row>
     <row r="707" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A707" s="2" t="s">
-        <v>1025</v>
+        <v>1023</v>
       </c>
       <c r="B707" s="2">
-        <v>1991</v>
+        <v>1993</v>
       </c>
       <c r="C707" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="D707" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
     </row>
     <row r="708" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A708" s="2" t="s">
-        <v>1026</v>
+        <v>1024</v>
       </c>
       <c r="B708" s="2">
         <v>1994</v>
       </c>
       <c r="C708" s="2" t="s">
-        <v>83</v>
+        <v>47</v>
       </c>
       <c r="D708" s="2" t="s">
-        <v>1027</v>
+        <v>47</v>
       </c>
     </row>
     <row r="709" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A709" s="2" t="s">
-        <v>1028</v>
+        <v>1025</v>
       </c>
       <c r="B709" s="2">
-        <v>1994</v>
+        <v>1991</v>
       </c>
       <c r="C709" s="2" t="s">
-        <v>11</v>
+        <v>55</v>
       </c>
       <c r="D709" s="2" t="s">
-        <v>11</v>
+        <v>55</v>
       </c>
     </row>
     <row r="710" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A710" s="2" t="s">
-        <v>1029</v>
+        <v>1026</v>
       </c>
       <c r="B710" s="2">
-        <v>1995</v>
+        <v>1994</v>
       </c>
       <c r="C710" s="2" t="s">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="D710" s="2" t="s">
-        <v>1030</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="711" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A711" s="2" t="s">
-        <v>1031</v>
+        <v>1028</v>
       </c>
       <c r="B711" s="2">
-        <v>1993</v>
+        <v>1994</v>
       </c>
       <c r="C711" s="2" t="s">
-        <v>164</v>
+        <v>11</v>
       </c>
       <c r="D711" s="2" t="s">
-        <v>164</v>
+        <v>11</v>
       </c>
     </row>
     <row r="712" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A712" s="2" t="s">
-        <v>1032</v>
+        <v>1029</v>
       </c>
       <c r="B712" s="2">
-        <v>1993</v>
+        <v>1995</v>
       </c>
       <c r="C712" s="2" t="s">
-        <v>83</v>
+        <v>34</v>
       </c>
       <c r="D712" s="2" t="s">
-        <v>78</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="713" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A713" s="2" t="s">
-        <v>1033</v>
+        <v>1031</v>
       </c>
       <c r="B713" s="2">
-        <v>1995</v>
+        <v>1993</v>
       </c>
       <c r="C713" s="2" t="s">
-        <v>108</v>
+        <v>164</v>
       </c>
       <c r="D713" s="2" t="s">
-        <v>99</v>
+        <v>164</v>
       </c>
     </row>
     <row r="714" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A714" s="2" t="s">
-        <v>1034</v>
+        <v>1032</v>
       </c>
       <c r="B714" s="2">
-        <v>1994</v>
+        <v>1993</v>
       </c>
       <c r="C714" s="2" t="s">
-        <v>108</v>
+        <v>83</v>
       </c>
       <c r="D714" s="2" t="s">
-        <v>1035</v>
+        <v>78</v>
       </c>
     </row>
     <row r="715" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A715" s="2" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="B715" s="2">
-        <v>1994</v>
+        <v>1995</v>
       </c>
       <c r="C715" s="2" t="s">
-        <v>65</v>
+        <v>108</v>
       </c>
       <c r="D715" s="2" t="s">
-        <v>20</v>
+        <v>99</v>
       </c>
     </row>
     <row r="716" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A716" s="2" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="B716" s="2">
         <v>1994</v>
       </c>
       <c r="C716" s="2" t="s">
-        <v>132</v>
+        <v>108</v>
       </c>
       <c r="D716" s="2" t="s">
-        <v>491</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="717" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A717" s="2" t="s">
-        <v>1038</v>
+        <v>1036</v>
       </c>
       <c r="B717" s="2">
-        <v>1995</v>
+        <v>1994</v>
       </c>
       <c r="C717" s="2" t="s">
-        <v>1039</v>
+        <v>65</v>
       </c>
       <c r="D717" s="2" t="s">
-        <v>1039</v>
+        <v>20</v>
       </c>
     </row>
     <row r="718" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A718" s="2" t="s">
-        <v>1040</v>
+        <v>1037</v>
       </c>
       <c r="B718" s="2">
-        <v>1996</v>
+        <v>1994</v>
       </c>
       <c r="C718" s="2" t="s">
-        <v>1039</v>
+        <v>132</v>
       </c>
       <c r="D718" s="2" t="s">
-        <v>1039</v>
+        <v>491</v>
       </c>
     </row>
     <row r="719" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A719" s="2" t="s">
-        <v>1041</v>
+        <v>1038</v>
       </c>
       <c r="B719" s="2">
-        <v>1994</v>
+        <v>1995</v>
       </c>
       <c r="C719" s="2" t="s">
-        <v>83</v>
+        <v>1039</v>
       </c>
       <c r="D719" s="2" t="s">
-        <v>1042</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="720" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A720" s="2" t="s">
-        <v>1043</v>
+        <v>1040</v>
       </c>
       <c r="B720" s="2">
-        <v>1995</v>
+        <v>1996</v>
       </c>
       <c r="C720" s="2" t="s">
-        <v>431</v>
+        <v>1039</v>
       </c>
       <c r="D720" s="2" t="s">
-        <v>15</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="721" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A721" s="2" t="s">
-        <v>1044</v>
+        <v>1041</v>
       </c>
       <c r="B721" s="2">
-        <v>1992</v>
+        <v>1994</v>
       </c>
       <c r="C721" s="2" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="D721" s="2" t="s">
-        <v>95</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="722" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A722" s="2" t="s">
-        <v>1045</v>
+        <v>1043</v>
       </c>
       <c r="B722" s="2">
         <v>1995</v>
       </c>
       <c r="C722" s="2" t="s">
-        <v>11</v>
+        <v>431</v>
       </c>
       <c r="D722" s="2" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
     </row>
     <row r="723" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A723" s="2" t="s">
-        <v>1046</v>
+        <v>1044</v>
       </c>
       <c r="B723" s="2">
-        <v>1995</v>
+        <v>1992</v>
       </c>
       <c r="C723" s="2" t="s">
-        <v>477</v>
+        <v>95</v>
       </c>
       <c r="D723" s="2" t="s">
-        <v>477</v>
+        <v>95</v>
       </c>
     </row>
     <row r="724" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A724" s="2" t="s">
-        <v>1047</v>
+        <v>1045</v>
       </c>
       <c r="B724" s="2">
-        <v>1993</v>
+        <v>1995</v>
       </c>
       <c r="C724" s="2" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="D724" s="2" t="s">
-        <v>152</v>
+        <v>11</v>
       </c>
     </row>
     <row r="725" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A725" s="2" t="s">
-        <v>1048</v>
+        <v>1046</v>
       </c>
       <c r="B725" s="2">
-        <v>1994</v>
+        <v>1995</v>
       </c>
       <c r="C725" s="2" t="s">
-        <v>579</v>
+        <v>477</v>
       </c>
       <c r="D725" s="2" t="s">
-        <v>221</v>
+        <v>477</v>
       </c>
     </row>
     <row r="726" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A726" s="2" t="s">
-        <v>1049</v>
+        <v>1047</v>
       </c>
       <c r="B726" s="2">
-        <v>1995</v>
+        <v>1993</v>
       </c>
       <c r="C726" s="2" t="s">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="D726" s="2" t="s">
-        <v>228</v>
+        <v>152</v>
       </c>
     </row>
     <row r="727" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A727" s="2" t="s">
-        <v>1050</v>
+        <v>1048</v>
       </c>
       <c r="B727" s="2">
-        <v>1993</v>
+        <v>1994</v>
       </c>
       <c r="C727" s="2" t="s">
-        <v>405</v>
+        <v>579</v>
       </c>
       <c r="D727" s="2" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
     </row>
     <row r="728" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A728" s="2" t="s">
-        <v>1051</v>
+        <v>1049</v>
       </c>
       <c r="B728" s="2">
-        <v>1992</v>
+        <v>1995</v>
       </c>
       <c r="C728" s="2" t="s">
-        <v>179</v>
+        <v>12</v>
       </c>
       <c r="D728" s="2" t="s">
-        <v>63</v>
+        <v>228</v>
       </c>
     </row>
     <row r="729" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A729" s="2" t="s">
-        <v>1052</v>
+        <v>1050</v>
       </c>
       <c r="B729" s="2">
-        <v>1994</v>
+        <v>1993</v>
       </c>
       <c r="C729" s="2" t="s">
-        <v>179</v>
+        <v>405</v>
       </c>
       <c r="D729" s="2" t="s">
-        <v>63</v>
+        <v>228</v>
       </c>
     </row>
     <row r="730" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A730" s="2" t="s">
-        <v>1053</v>
+        <v>1051</v>
       </c>
       <c r="B730" s="2">
-        <v>1993</v>
+        <v>1992</v>
       </c>
       <c r="C730" s="2" t="s">
-        <v>405</v>
+        <v>179</v>
       </c>
       <c r="D730" s="2" t="s">
-        <v>467</v>
+        <v>63</v>
       </c>
     </row>
     <row r="731" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A731" s="2" t="s">
-        <v>1054</v>
+        <v>1052</v>
       </c>
       <c r="B731" s="2">
-        <v>1992</v>
+        <v>1994</v>
       </c>
       <c r="C731" s="2" t="s">
-        <v>12</v>
+        <v>179</v>
       </c>
       <c r="D731" s="2" t="s">
-        <v>12</v>
+        <v>63</v>
       </c>
     </row>
     <row r="732" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A732" s="2" t="s">
-        <v>1055</v>
+        <v>1053</v>
       </c>
       <c r="B732" s="2">
-        <v>1996</v>
+        <v>1993</v>
       </c>
       <c r="C732" s="2" t="s">
-        <v>80</v>
+        <v>405</v>
       </c>
       <c r="D732" s="2" t="s">
-        <v>662</v>
+        <v>467</v>
       </c>
     </row>
     <row r="733" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A733" s="2" t="s">
-        <v>1056</v>
+        <v>1054</v>
       </c>
       <c r="B733" s="2">
-        <v>1995</v>
+        <v>1992</v>
       </c>
       <c r="C733" s="2" t="s">
-        <v>279</v>
+        <v>12</v>
       </c>
       <c r="D733" s="2" t="s">
-        <v>221</v>
+        <v>12</v>
       </c>
     </row>
     <row r="734" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A734" s="2" t="s">
-        <v>1057</v>
+        <v>1055</v>
       </c>
       <c r="B734" s="2">
-        <v>1995</v>
+        <v>1996</v>
       </c>
       <c r="C734" s="2" t="s">
-        <v>207</v>
+        <v>80</v>
       </c>
       <c r="D734" s="2" t="s">
-        <v>207</v>
+        <v>662</v>
       </c>
     </row>
     <row r="735" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A735" s="2" t="s">
-        <v>1058</v>
+        <v>1056</v>
       </c>
       <c r="B735" s="2">
-        <v>1994</v>
+        <v>1995</v>
       </c>
       <c r="C735" s="2" t="s">
-        <v>166</v>
+        <v>279</v>
       </c>
       <c r="D735" s="2" t="s">
-        <v>489</v>
+        <v>221</v>
       </c>
     </row>
     <row r="736" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A736" s="2" t="s">
-        <v>1059</v>
+        <v>1057</v>
       </c>
       <c r="B736" s="2">
-        <v>1996</v>
+        <v>1995</v>
       </c>
       <c r="C736" s="2" t="s">
-        <v>1020</v>
+        <v>207</v>
       </c>
       <c r="D736" s="2" t="s">
-        <v>1060</v>
+        <v>207</v>
       </c>
     </row>
     <row r="737" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A737" s="2" t="s">
-        <v>1061</v>
+        <v>1058</v>
       </c>
       <c r="B737" s="2">
-        <v>1992</v>
+        <v>1994</v>
       </c>
       <c r="C737" s="2" t="s">
-        <v>52</v>
+        <v>166</v>
       </c>
       <c r="D737" s="2" t="s">
-        <v>580</v>
+        <v>489</v>
       </c>
     </row>
     <row r="738" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A738" s="2" t="s">
-        <v>1062</v>
+        <v>1059</v>
       </c>
       <c r="B738" s="2">
-        <v>1993</v>
+        <v>1996</v>
       </c>
       <c r="C738" s="2" t="s">
-        <v>52</v>
+        <v>1020</v>
       </c>
       <c r="D738" s="2" t="s">
-        <v>580</v>
+        <v>1060</v>
       </c>
     </row>
     <row r="739" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A739" s="2" t="s">
-        <v>1063</v>
+        <v>1061</v>
       </c>
       <c r="B739" s="2">
         <v>1992</v>
       </c>
       <c r="C739" s="2" t="s">
-        <v>12</v>
+        <v>52</v>
       </c>
       <c r="D739" s="2" t="s">
-        <v>12</v>
+        <v>580</v>
       </c>
     </row>
     <row r="740" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A740" s="2" t="s">
-        <v>1064</v>
+        <v>1062</v>
       </c>
       <c r="B740" s="2">
-        <v>1996</v>
+        <v>1993</v>
       </c>
       <c r="C740" s="2" t="s">
-        <v>83</v>
+        <v>52</v>
       </c>
       <c r="D740" s="2" t="s">
-        <v>257</v>
+        <v>580</v>
       </c>
     </row>
     <row r="741" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A741" s="2" t="s">
-        <v>1065</v>
+        <v>1063</v>
       </c>
       <c r="B741" s="2">
-        <v>1994</v>
+        <v>1992</v>
       </c>
       <c r="C741" s="2" t="s">
-        <v>364</v>
+        <v>12</v>
       </c>
       <c r="D741" s="2" t="s">
-        <v>177</v>
+        <v>12</v>
       </c>
     </row>
     <row r="742" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A742" s="2" t="s">
-        <v>1066</v>
+        <v>1064</v>
       </c>
       <c r="B742" s="2">
-        <v>1993</v>
+        <v>1996</v>
       </c>
       <c r="C742" s="2" t="s">
-        <v>331</v>
+        <v>83</v>
       </c>
       <c r="D742" s="2" t="s">
-        <v>489</v>
+        <v>257</v>
       </c>
     </row>
     <row r="743" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A743" s="2" t="s">
-        <v>1067</v>
+        <v>1065</v>
       </c>
       <c r="B743" s="2">
         <v>1994</v>
       </c>
       <c r="C743" s="2" t="s">
-        <v>55</v>
+        <v>364</v>
       </c>
       <c r="D743" s="2" t="s">
-        <v>81</v>
+        <v>177</v>
       </c>
     </row>
     <row r="744" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A744" s="2" t="s">
-        <v>1068</v>
+        <v>1066</v>
       </c>
       <c r="B744" s="2">
         <v>1993</v>
       </c>
       <c r="C744" s="2" t="s">
-        <v>193</v>
+        <v>331</v>
       </c>
       <c r="D744" s="2" t="s">
-        <v>224</v>
+        <v>489</v>
       </c>
     </row>
     <row r="745" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A745" s="2" t="s">
-        <v>1069</v>
+        <v>1067</v>
       </c>
       <c r="B745" s="2">
         <v>1994</v>
       </c>
       <c r="C745" s="2" t="s">
-        <v>482</v>
+        <v>55</v>
       </c>
       <c r="D745" s="2" t="s">
-        <v>1070</v>
+        <v>81</v>
       </c>
     </row>
     <row r="746" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A746" s="2" t="s">
-        <v>1071</v>
+        <v>1068</v>
       </c>
       <c r="B746" s="2">
-        <v>1994</v>
+        <v>1993</v>
       </c>
       <c r="C746" s="2" t="s">
-        <v>431</v>
+        <v>193</v>
       </c>
       <c r="D746" s="2" t="s">
-        <v>395</v>
+        <v>224</v>
       </c>
     </row>
     <row r="747" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A747" s="2" t="s">
-        <v>1072</v>
+        <v>1069</v>
       </c>
       <c r="B747" s="2">
-        <v>1992</v>
+        <v>1994</v>
       </c>
       <c r="C747" s="2" t="s">
-        <v>166</v>
+        <v>482</v>
       </c>
       <c r="D747" s="2" t="s">
-        <v>336</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="748" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A748" s="2" t="s">
-        <v>1073</v>
+        <v>1071</v>
       </c>
       <c r="B748" s="2">
-        <v>1993</v>
+        <v>1994</v>
       </c>
       <c r="C748" s="2" t="s">
-        <v>482</v>
+        <v>431</v>
       </c>
       <c r="D748" s="2" t="s">
-        <v>1074</v>
+        <v>395</v>
       </c>
     </row>
     <row r="749" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A749" s="2" t="s">
-        <v>1075</v>
+        <v>1072</v>
       </c>
       <c r="B749" s="2">
-        <v>1994</v>
+        <v>1992</v>
       </c>
       <c r="C749" s="2" t="s">
-        <v>1076</v>
+        <v>166</v>
       </c>
       <c r="D749" s="2" t="s">
-        <v>714</v>
+        <v>336</v>
       </c>
     </row>
     <row r="750" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A750" s="2" t="s">
-        <v>1077</v>
+        <v>1073</v>
       </c>
       <c r="B750" s="2">
-        <v>1994</v>
+        <v>1993</v>
       </c>
       <c r="C750" s="2" t="s">
-        <v>364</v>
+        <v>482</v>
       </c>
       <c r="D750" s="2" t="s">
-        <v>177</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="751" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A751" s="2" t="s">
-        <v>1078</v>
+        <v>1075</v>
       </c>
       <c r="B751" s="2">
-        <v>1993</v>
+        <v>1994</v>
       </c>
       <c r="C751" s="2" t="s">
-        <v>19</v>
+        <v>1076</v>
       </c>
       <c r="D751" s="2" t="s">
-        <v>19</v>
+        <v>714</v>
       </c>
     </row>
     <row r="752" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A752" s="2" t="s">
-        <v>1079</v>
+        <v>1077</v>
       </c>
       <c r="B752" s="2">
         <v>1994</v>
       </c>
       <c r="C752" s="2" t="s">
-        <v>494</v>
+        <v>364</v>
       </c>
       <c r="D752" s="2" t="s">
-        <v>1080</v>
+        <v>177</v>
       </c>
     </row>
     <row r="753" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A753" s="2" t="s">
-        <v>1081</v>
+        <v>1078</v>
       </c>
       <c r="B753" s="2">
-        <v>1992</v>
+        <v>1993</v>
       </c>
       <c r="C753" s="2" t="s">
-        <v>52</v>
+        <v>19</v>
       </c>
       <c r="D753" s="2" t="s">
-        <v>483</v>
+        <v>19</v>
       </c>
     </row>
     <row r="754" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A754" s="2" t="s">
-        <v>1082</v>
+        <v>1079</v>
       </c>
       <c r="B754" s="2">
-        <v>1995</v>
+        <v>1994</v>
       </c>
       <c r="C754" s="2" t="s">
-        <v>193</v>
+        <v>494</v>
       </c>
       <c r="D754" s="2" t="s">
-        <v>1083</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="755" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A755" s="2" t="s">
-        <v>1084</v>
+        <v>1081</v>
       </c>
       <c r="B755" s="2">
-        <v>1996</v>
+        <v>1992</v>
       </c>
       <c r="C755" s="2" t="s">
-        <v>11</v>
+        <v>52</v>
       </c>
       <c r="D755" s="2" t="s">
-        <v>1085</v>
+        <v>483</v>
       </c>
     </row>
     <row r="756" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A756" s="2" t="s">
-        <v>1086</v>
+        <v>1082</v>
       </c>
       <c r="B756" s="2">
-        <v>1992</v>
+        <v>1995</v>
       </c>
       <c r="C756" s="2" t="s">
-        <v>431</v>
+        <v>193</v>
       </c>
       <c r="D756" s="2" t="s">
-        <v>204</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="757" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A757" s="2" t="s">
-        <v>1087</v>
+        <v>1084</v>
       </c>
       <c r="B757" s="2">
-        <v>1993</v>
+        <v>1996</v>
       </c>
       <c r="C757" s="2" t="s">
-        <v>431</v>
+        <v>11</v>
       </c>
       <c r="D757" s="2" t="s">
-        <v>204</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="758" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A758" s="2" t="s">
-        <v>1088</v>
+        <v>1086</v>
       </c>
       <c r="B758" s="2">
-        <v>1994</v>
+        <v>1992</v>
       </c>
       <c r="C758" s="2" t="s">
-        <v>108</v>
+        <v>431</v>
       </c>
       <c r="D758" s="2" t="s">
         <v>204</v>
@@ -14269,13 +14275,13 @@
     </row>
     <row r="759" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A759" s="2" t="s">
-        <v>1089</v>
+        <v>1087</v>
       </c>
       <c r="B759" s="2">
-        <v>1995</v>
+        <v>1993</v>
       </c>
       <c r="C759" s="2" t="s">
-        <v>108</v>
+        <v>431</v>
       </c>
       <c r="D759" s="2" t="s">
         <v>204</v>
@@ -14283,169 +14289,197 @@
     </row>
     <row r="760" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A760" s="2" t="s">
-        <v>1090</v>
+        <v>1088</v>
       </c>
       <c r="B760" s="2">
-        <v>1992</v>
+        <v>1994</v>
       </c>
       <c r="C760" s="2" t="s">
-        <v>265</v>
+        <v>108</v>
       </c>
       <c r="D760" s="2" t="s">
-        <v>265</v>
+        <v>204</v>
       </c>
     </row>
     <row r="761" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A761" s="2" t="s">
-        <v>1091</v>
+        <v>1089</v>
       </c>
       <c r="B761" s="2">
-        <v>1994</v>
+        <v>1995</v>
       </c>
       <c r="C761" s="2" t="s">
-        <v>59</v>
+        <v>108</v>
       </c>
       <c r="D761" s="2" t="s">
-        <v>957</v>
+        <v>204</v>
       </c>
     </row>
     <row r="762" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A762" s="2" t="s">
-        <v>1092</v>
+        <v>1090</v>
       </c>
       <c r="B762" s="2">
-        <v>1994</v>
+        <v>1992</v>
       </c>
       <c r="C762" s="2" t="s">
-        <v>55</v>
+        <v>265</v>
       </c>
       <c r="D762" s="2" t="s">
-        <v>55</v>
+        <v>265</v>
       </c>
     </row>
     <row r="763" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A763" s="2" t="s">
-        <v>1093</v>
+        <v>1091</v>
       </c>
       <c r="B763" s="2">
-        <v>1992</v>
+        <v>1994</v>
       </c>
       <c r="C763" s="2" t="s">
-        <v>294</v>
+        <v>59</v>
       </c>
       <c r="D763" s="2" t="s">
-        <v>294</v>
+        <v>957</v>
       </c>
     </row>
     <row r="764" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A764" s="2" t="s">
-        <v>1094</v>
+        <v>1092</v>
       </c>
       <c r="B764" s="2">
-        <v>1993</v>
+        <v>1994</v>
       </c>
       <c r="C764" s="2" t="s">
-        <v>336</v>
+        <v>55</v>
       </c>
       <c r="D764" s="2" t="s">
-        <v>336</v>
+        <v>55</v>
       </c>
     </row>
     <row r="765" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A765" s="2" t="s">
-        <v>1095</v>
+        <v>1093</v>
       </c>
       <c r="B765" s="2">
-        <v>1993</v>
+        <v>1992</v>
       </c>
       <c r="C765" s="2" t="s">
-        <v>83</v>
+        <v>294</v>
       </c>
       <c r="D765" s="2" t="s">
-        <v>1042</v>
+        <v>294</v>
       </c>
     </row>
     <row r="766" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A766" s="2" t="s">
-        <v>1096</v>
+        <v>1094</v>
       </c>
       <c r="B766" s="2">
-        <v>1994</v>
+        <v>1993</v>
       </c>
       <c r="C766" s="2" t="s">
-        <v>193</v>
+        <v>336</v>
       </c>
       <c r="D766" s="2" t="s">
-        <v>523</v>
+        <v>336</v>
       </c>
     </row>
     <row r="767" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A767" s="2" t="s">
-        <v>1097</v>
+        <v>1095</v>
       </c>
       <c r="B767" s="2">
-        <v>1992</v>
+        <v>1993</v>
       </c>
       <c r="C767" s="2" t="s">
-        <v>111</v>
+        <v>83</v>
       </c>
       <c r="D767" s="2" t="s">
-        <v>946</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="768" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A768" s="2" t="s">
-        <v>1098</v>
+        <v>1096</v>
       </c>
       <c r="B768" s="2">
         <v>1994</v>
       </c>
       <c r="C768" s="2" t="s">
-        <v>19</v>
+        <v>193</v>
       </c>
       <c r="D768" s="2" t="s">
-        <v>44</v>
+        <v>523</v>
       </c>
     </row>
     <row r="769" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A769" s="2" t="s">
-        <v>1099</v>
+        <v>1097</v>
       </c>
       <c r="B769" s="2">
-        <v>1993</v>
+        <v>1992</v>
       </c>
       <c r="C769" s="2" t="s">
-        <v>28</v>
+        <v>111</v>
       </c>
       <c r="D769" s="2" t="s">
-        <v>136</v>
+        <v>946</v>
       </c>
     </row>
     <row r="770" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A770" s="2" t="s">
-        <v>1100</v>
+        <v>1098</v>
       </c>
       <c r="B770" s="2">
-        <v>1993</v>
+        <v>1994</v>
       </c>
       <c r="C770" s="2" t="s">
-        <v>179</v>
+        <v>19</v>
       </c>
       <c r="D770" s="2" t="s">
-        <v>378</v>
+        <v>44</v>
       </c>
     </row>
     <row r="771" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A771" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="B771" s="2">
+        <v>1993</v>
+      </c>
+      <c r="C771" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D771" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="772" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A772" s="2" t="s">
+        <v>1100</v>
+      </c>
+      <c r="B772" s="2">
+        <v>1993</v>
+      </c>
+      <c r="C772" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="D772" s="2" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="773" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A773" s="2" t="s">
         <v>1101</v>
       </c>
-      <c r="B771" s="2">
+      <c r="B773" s="2">
         <v>1995</v>
       </c>
-      <c r="C771" s="2" t="s">
+      <c r="C773" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D771" s="2" t="s">
+      <c r="D773" s="2" t="s">
         <v>1102</v>
       </c>
     </row>
@@ -14467,7 +14501,7 @@
     <col min="6" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
         <v>1103</v>
       </c>

</xml_diff>